<commit_message>
Ship BalVoi:60 hourly cadence, preview mode, and publication safety.
Replace the twice-hourly BalVoi:30 flow with process-at-:51 / publish-at-:00 ownership windows, isolated real preview generation, concurrent language workers, and fail-closed validation without Megaphone or live metadata side effects.
</commit_message>
<xml_diff>
--- a/BalVoi_30 Content.xlsx
+++ b/BalVoi_30 Content.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JeffreyCrump\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft16340667-my.sharepoint.com/personal/nvithanala_newsgenie_ai/Documents/Desktop/BalVoi_30/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAEBA2F1-DA58-4F11-BE30-1915A801D1A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{CAEBA2F1-DA58-4F11-BE30-1915A801D1A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCC1C599-70E2-4D7E-8C9D-C286FBCB7CE0}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{04BEA111-B2D1-43D4-8D75-B7B3005C7E34}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="5" xr2:uid="{04BEA111-B2D1-43D4-8D75-B7B3005C7E34}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome" sheetId="7" r:id="rId1"/>
@@ -1382,260 +1382,260 @@
 Nasıl olduğunu öğrenmek için NewsGenie.ai adresini ziyaret edin.</t>
   </si>
   <si>
+    <t>English Ad 2</t>
+  </si>
+  <si>
+    <t>Spanish Ad 2</t>
+  </si>
+  <si>
+    <t>Portuguese Ad 2</t>
+  </si>
+  <si>
+    <t>French Ad 2</t>
+  </si>
+  <si>
+    <t>German Ad 2</t>
+  </si>
+  <si>
+    <t>Arabic Ad 2</t>
+  </si>
+  <si>
+    <t>Russian Ad 2</t>
+  </si>
+  <si>
+    <t>Turkish Ad 2</t>
+  </si>
+  <si>
+    <t>What does your brand stand for?
+In a world of information overload, growing polarization, and declining trust, consumers increasingly support organizations that value transparency, trust, and accountability.
+BalVoi:60 is building a global network of multilingual news programming powered by NewsGenie technology and dedicated to trustworthy information and informed audiences.
+We invite mission-driven brands to join us.
+If your organization believes technology should strengthen understanding rather than division, and that trust is earned through action, we'd love to talk.
+Learn more about sponsorship opportunities at BalVoi.com.
+BalVoi:60. Trustworthy information for a connected world.</t>
+  </si>
+  <si>
+    <t>¿Qué representa su marca?
+En un mundo de sobrecarga informativa, creciente polarización y disminución de la confianza, los consumidores apoyan cada vez más a las organizaciones que valoran la transparencia, la confianza y la responsabilidad.
+BalVoi:60 está construyendo una red global de programación informativa multilingüe impulsada por la tecnología de NewsGenie y dedicada a la información confiable y a audiencias bien informadas.
+Invitamos a las marcas con propósito a unirse a nosotros.
+Si su organización cree que la tecnología debe fortalecer el entendimiento en lugar de la división, y que la confianza se gana con acciones, nos gustaría conversar.
+Obtenga más información sobre oportunidades de patrocinio en BalVoi.com.
+BalVoi:60. Información confiable para un mundo conectado.</t>
+  </si>
+  <si>
+    <t>O que a sua marca representa?
+Em um mundo de excesso de informação, crescente polarização e queda da confiança, os consumidores apoiam cada vez mais organizações que valorizam transparência, confiança e responsabilidade.
+A BalVoi:60 está construindo uma rede global de programação informativa multilíngue impulsionada pela tecnologia da NewsGenie e dedicada à informação confiável e a públicos bem informados.
+Convidamos marcas com propósito a se juntarem a nós.
+Se sua organização acredita que a tecnologia deve fortalecer a compreensão em vez da divisão, e que a confiança é conquistada por meio de ações, gostaríamos de conversar.
+Saiba mais sobre oportunidades de patrocínio em BalVoi.com.
+BalVoi:60. Informação confiável para um mundo conectado.</t>
+  </si>
+  <si>
+    <t>Que représente votre marque ?
+Dans un monde marqué par la surcharge d'information, une polarisation croissante et un recul de la confiance, les consommateurs soutiennent de plus en plus les organisations qui valorisent la transparence, la confiance et la responsabilité.
+BalVoi:60 construit un réseau mondial de programmes d'information multilingues alimenté par la technologie NewsGenie et dédié à une information fiable et à des audiences éclairées.
+Nous invitons les marques porteuses d'une mission à nous rejoindre.
+Si votre organisation croit que la technologie doit renforcer la compréhension plutôt que la division, et que la confiance se gagne par les actes, nous serions heureux d'échanger avec vous.
+Découvrez les opportunités de partenariat sur BalVoi.com.
+BalVoi:60. Une information fiable pour un monde connecté.</t>
+  </si>
+  <si>
+    <t>Wofür steht Ihre Marke?
+In einer Welt voller Informationsüberlastung, wachsender Polarisierung und schwindenden Vertrauens unterstützen Verbraucher zunehmend Organisationen, die Transparenz, Vertrauen und Verantwortung schätzen.
+BalVoi:60 baut ein globales Netzwerk mehrsprachiger Nachrichtenprogramme auf, das von der NewsGenie-Technologie unterstützt wird und sich vertrauenswürdigen Informationen sowie informierten Zielgruppen widmet.
+Wir laden werteorientierte Marken ein, Teil dieser Mission zu werden.
+Wenn Ihr Unternehmen daran glaubt, dass Technologie Verständnis fördern statt Spaltung vertiefen sollte und dass Vertrauen durch Taten verdient wird, würden wir uns gerne mit Ihnen austauschen.
+Erfahren Sie mehr über Sponsoring-Möglichkeiten auf BalVoi.com.
+BalVoi:60. Vertrauenswürdige Informationen für eine vernetzte Welt.</t>
+  </si>
+  <si>
+    <t>بماذا تُعرف علامتكم التجارية؟
+في عالم يشهد فيضًا من المعلومات وتزايدًا في الاستقطاب وتراجعًا في الثقة، يتجه المستهلكون بشكل متزايد نحو المؤسسات التي تؤمن بالشفافية والثقة والمساءلة.
+تبني BalVoi:60 شبكة عالمية من البرامج الإخبارية متعددة اللغات، مدعومة بتقنية NewsGenie ومكرسة لتقديم معلومات موثوقة لجمهور واعٍ ومطلع.
+ندعو العلامات التجارية ذات الرسالة الواضحة للانضمام إلينا.
+إذا كانت مؤسستكم تؤمن بأن التكنولوجيا يجب أن تعزز الفهم بدلاً من الانقسام، وأن الثقة تُكتسب من خلال الأفعال، فسيسعدنا التواصل معكم.
+تعرفوا على فرص الرعاية عبر BalVoi.com.
+BalVoi:60. معلومات موثوقة لعالم مترابط.</t>
+  </si>
+  <si>
+    <t>Что представляет собой ваш бренд?
+В мире информационной перегрузки, растущей поляризации и снижения уровня доверия люди всё чаще поддерживают организации, которые ценят прозрачность, доверие и ответственность.
+BalVoi:60 создаёт глобальную сеть многоязычных новостных программ на базе технологий NewsGenie, ориентированную на надёжную информацию и информированную аудиторию.
+Мы приглашаем бренды с миссией присоединиться к нам.
+Если ваша организация считает, что технологии должны укреплять взаимопонимание, а не усиливать разногласия, и что доверие заслуживается действиями, мы будем рады сотрудничеству.
+Узнайте больше о возможностях спонсорства на BalVoi.com.
+BalVoi:60. Надёжная информация для взаимосвязанного мира.</t>
+  </si>
+  <si>
+    <t>Markanız neyi temsil ediyor?
+Bilgi fazlalığının, artan kutuplaşmanın ve azalan güvenin yaşandığı bir dünyada, tüketiciler şeffaflık, güven ve hesap verebilirlik değerlerini benimseyen kuruluşları giderek daha fazla desteklemektedir.
+BalVoi:60, NewsGenie teknolojisiyle desteklenen ve güvenilir bilgi ile bilinçli kitlelere odaklanan çok dilli küresel bir haber ağı inşa etmektedir.
+Misyon sahibi markaları bize katılmaya davet ediyoruz.
+Kuruluşunuz teknolojinin ayrışmayı değil anlayışı güçlendirmesi gerektiğine ve güvenin eylemlerle kazanıldığına inanıyorsa, sizinle konuşmak isteriz.
+Sponsorluk fırsatları hakkında daha fazla bilgi için BalVoi.com'u ziyaret edin.
+BalVoi:60. Bağlantılı bir dünya için güvenilir bilgi.</t>
+  </si>
+  <si>
+    <t>Artificial intelligence is changing how the world creates, distributes, and consumes information.
+The question is not whether AI will shape the future.
+The question is how.
+BalVoi:60 partners with organizations that believe AI can be used responsibly to increase transparency, improve understanding, and strengthen public trust.
+Our multilingual information network reaches audiences across North America, Latin America, Europe, the Middle East, and Eurasia.
+If your brand believes in innovation with purpose, we invite you to join us.
+BalVoi:60.
+Global reach. Trustworthy information. Responsible AI.</t>
+  </si>
+  <si>
+    <t>La inteligencia artificial está transformando la forma en que el mundo crea, distribuye y consume información.
+La pregunta no es si la inteligencia artificial cambiará el futuro.
+La pregunta es cómo lo hará.
+BalVoi:60 colabora con organizaciones que creen que la inteligencia artificial puede utilizarse de manera responsable para aumentar la transparencia, mejorar el entendimiento y fortalecer la confianza pública.
+Nuestra red multilingüe de información conecta audiencias en América del Norte, América Latina, Europa, Oriente Medio y Eurasia.
+Si su organización cree en la innovación con propósito, queremos conocerla.
+BalVoi:60.
+Alcance global. Información confiable. Inteligencia artificial responsable.</t>
+  </si>
+  <si>
+    <t>A inteligência artificial está transformando a maneira como o mundo cria, distribui e consome informação.
+A questão não é se a inteligência artificial moldará o futuro.
+A questão é como.
+A BalVoi:60 trabalha com organizações que acreditam que a inteligência artificial pode ser usada de forma responsável para aumentar a transparência, melhorar a compreensão e fortalecer a confiança pública.
+Nossa rede multilíngue de informação conecta audiências na América do Norte, América Latina, Europa, Oriente Médio e Eurásia.
+Se sua organização acredita em inovação com propósito, queremos conversar.
+BalVoi:60.
+Alcance global. Informação confiável. Inteligência artificial responsável.</t>
+  </si>
+  <si>
+    <t>L'intelligence artificielle transforme la manière dont le monde crée, diffuse et consomme l'information.
+La question n'est pas de savoir si l'intelligence artificielle façonnera l'avenir.
+La question est de savoir comment.
+BalVoi:60 s'associe à des organisations qui croient que l'intelligence artificielle peut être utilisée de manière responsable pour renforcer la transparence, améliorer la compréhension et accroître la confiance du public.
+Notre réseau multilingue d'information rejoint des audiences en Amérique du Nord, en Amérique latine, en Europe, au Moyen-Orient et en Eurasie.
+Si votre organisation croit en une innovation porteuse de sens, nous aimerions échanger avec vous.
+BalVoi:60.
+Portée mondiale. Information digne de confiance. Intelligence artificielle responsable.</t>
+  </si>
+  <si>
+    <t>Künstliche Intelligenz verändert, wie die Welt Informationen erstellt, verbreitet und konsumiert.
+Die Frage ist nicht, ob künstliche Intelligenz die Zukunft prägen wird.
+Die Frage ist, wie.
+BalVoi:60 arbeitet mit Organisationen zusammen, die daran glauben, dass künstliche Intelligenz verantwortungsvoll eingesetzt werden kann, um Transparenz zu fördern, Verständnis zu verbessern und öffentliches Vertrauen zu stärken.
+Unser mehrsprachiges Informationsnetzwerk erreicht Zielgruppen in Nordamerika, Lateinamerika, Europa, dem Nahen Osten und Eurasien.
+Wenn Ihr Unternehmen an Innovation mit Verantwortung glaubt, würden wir gerne mit Ihnen sprechen.
+BalVoi:60.
+Globale Reichweite. Vertrauenswürdige Informationen. Verantwortungsvolle künstliche Intelligenz.</t>
+  </si>
+  <si>
+    <t>يُغيّر الذكاء الاصطناعي الطريقة التي يُنشئ بها العالم المعلومات ويوزعها ويستهلكها.
+السؤال ليس ما إذا كان الذكاء الاصطناعي سيشكل المستقبل.
+السؤال هو كيف.
+تتعاون BalVoi:60 مع المؤسسات التي تؤمن بأن الذكاء الاصطناعي يمكن استخدامه بمسؤولية لتعزيز الشفافية وتحسين الفهم وتقوية الثقة العامة.
+تصل شبكتنا متعددة اللغات للمعلومات إلى جماهير في أمريكا الشمالية وأمريكا اللاتينية وأوروبا والشرق الأوسط وأوراسيا.
+إذا كانت مؤسستكم تؤمن بالابتكار الهادف، فنحن ندعوكم للانضمام إلينا.
+BalVoi:60.
+انتشار عالمي. معلومات جديرة بالثقة. ذكاء اصطناعي مسؤول.</t>
+  </si>
+  <si>
+    <t>Искусственный интеллект меняет способы создания, распространения и потребления информации во всём мире.
+Вопрос не в том, повлияет ли искусственный интеллект на будущее.
+Вопрос в том, каким будет это влияние.
+BalVoi:60 сотрудничает с организациями, которые считают, что искусственный интеллект должен использоваться ответственно для повышения прозрачности, улучшения понимания происходящего и укрепления общественного доверия.
+Наша многоязычная информационная сеть объединяет аудитории в Северной Америке, Латинской Америке, Европе, на Ближнем Востоке и в Евразии.
+Если ваша организация верит в инновации со смыслом, мы будем рады сотрудничеству.
+BalVoi:60.
+Глобальный охват. Надёжная информация. Ответственный искусственный интеллект.</t>
+  </si>
+  <si>
+    <t>Yapay zekâ, dünyanın bilgiyi üretme, dağıtma ve tüketme biçimini değiştiriyor.
+Soru, yapay zekânın geleceği şekillendirip şekillendirmeyeceği değildir.
+Soru, bunu nasıl yapacağıdır.
+BalVoi:60; yapay zekânın şeffaflığı artırmak, anlayışı geliştirmek ve kamu güvenini güçlendirmek için sorumlu bir şekilde kullanılabileceğine inanan kuruluşlarla iş birliği yapmaktadır.
+Çok dilli bilgi ağımız Kuzey Amerika, Latin Amerika, Avrupa, Orta Doğu ve Avrasya'daki kitlelere ulaşmaktadır.
+Kuruluşunuz amaç odaklı inovasyona inanıyorsa, sizinle tanışmak isteriz.
+BalVoi:60.
+Küresel erişim. Güvenilir bilgi. Sorumlu yapay zekâ.</t>
+  </si>
+  <si>
     <t>Every day, millions of people are exposed to more information than any generation before them.
 Trust has never been more valuable.
-BalVoi:30 delivers balanced and trustworthy news updates to a growing global audience every thirty minutes across multiple languages and regions.
-For brands committed to integrity, transparency, innovation, and responsible AI, BalVoi:30 offers more than advertising.
+BalVoi:60 delivers balanced and trustworthy news updates to a growing global audience every sixty minutes across multiple languages and regions.
+For brands committed to integrity, transparency, innovation, and responsible AI, BalVoi:60 offers more than advertising.
 It offers alignment with values.
 Reach audiences who value facts, thoughtful analysis, and trustworthy information.
 To learn more about sponsorship opportunities, visit BalVoi.com.
-BalVoi:30. The balanced voice in news.</t>
+BalVoi:60. The balanced voice in news.</t>
   </si>
   <si>
     <t>Cada día, millones de personas están expuestas a más información que cualquier generación anterior.
 La confianza nunca ha sido tan valiosa.
-BalVoi:30 ofrece noticias equilibradas y confiables a una audiencia global en crecimiento, con actualizaciones cada treinta minutos en múltiples idiomas y regiones.
-Para las marcas comprometidas con la integridad, la transparencia, la innovación y la inteligencia artificial responsable, BalVoi:30 ofrece mucho más que publicidad.
+BalVoi:60 ofrece noticias equilibradas y confiables a una audiencia global en crecimiento, con actualizaciones cada sesenta minutos en múltiples idiomas y regiones.
+Para las marcas comprometidas con la integridad, la transparencia, la innovación y la inteligencia artificial responsable, BalVoi:60 ofrece mucho más que publicidad.
 Ofrece una conexión con valores compartidos.
 Conecte con audiencias que valoran los hechos, el análisis reflexivo y la información confiable.
 Para conocer oportunidades de patrocinio, visite BalVoi.com.
-BalVoi:30. La voz equilibrada de las noticias.</t>
+BalVoi:60. La voz equilibrada de las noticias.</t>
   </si>
   <si>
     <t>Todos os dias, milhões de pessoas são expostas a mais informação do que qualquer geração anterior.
 A confiança nunca foi tão valiosa.
-A BalVoi:30 oferece notícias equilibradas e confiáveis para uma audiência global em crescimento, com atualizações a cada trinta minutos em vários idiomas e regiões.
-Para marcas comprometidas com integridade, transparência, inovação e inteligência artificial responsável, a BalVoi:30 oferece mais do que publicidade.
+A BalVoi:60 oferece notícias equilibradas e confiáveis para uma audiência global em crescimento, com atualizações a cada sessenta minutos em vários idiomas e regiões.
+Para marcas comprometidas com integridade, transparência, inovação e inteligência artificial responsável, a BalVoi:60 oferece mais do que publicidade.
 Oferece alinhamento com valores.
 Conecte-se com públicos que valorizam fatos, análises cuidadosas e informação confiável.
 Saiba mais sobre oportunidades de patrocínio em BalVoi.com.
-BalVoi:30. A voz equilibrada das notícias.</t>
+BalVoi:60. A voz equilibrada das notícias.</t>
   </si>
   <si>
     <t>Chaque jour, des millions de personnes sont exposées à davantage d'informations que n'importe quelle génération avant elles.
 La confiance n'a jamais eu autant de valeur.
-BalVoi:30 propose des actualités équilibrées et dignes de confiance à une audience mondiale en pleine croissance, avec des mises à jour toutes les trente minutes dans plusieurs langues et régions.
-Pour les marques qui valorisent l'intégrité, la transparence, l'innovation et une intelligence artificielle responsable, BalVoi:30 représente bien plus qu'un espace publicitaire.
+BalVoi:60 propose des actualités équilibrées et dignes de confiance à une audience mondiale en pleine croissance, avec des mises à jour toutes les soixante minutes dans plusieurs langues et régions.
+Pour les marques qui valorisent l'intégrité, la transparence, l'innovation et une intelligence artificielle responsable, BalVoi:60 représente bien plus qu'un espace publicitaire.
 C'est l'occasion de s'associer à des valeurs partagées.
 Rejoignez des audiences qui apprécient les faits, l'analyse réfléchie et une information digne de confiance.
 Pour en savoir plus sur les opportunités de partenariat, rendez-vous sur BalVoi.com.
-BalVoi:30. La voix équilibrée de l'actualité.</t>
+BalVoi:60. La voix équilibrée de l'actualité.</t>
   </si>
   <si>
     <t>Jeden Tag werden Millionen Menschen mit mehr Informationen konfrontiert als jede Generation zuvor.
 Vertrauen war noch nie so wertvoll.
-BalVoi:30 liefert ausgewogene und vertrauenswürdige Nachrichten an ein wachsendes globales Publikum – alle dreißig Minuten, in mehreren Sprachen und Regionen.
-Für Marken, die für Integrität, Transparenz, Innovation und verantwortungsvolle künstliche Intelligenz stehen, bietet BalVoi:30 mehr als Werbung.
+BalVoi:60 liefert ausgewogene und vertrauenswürdige Nachrichten an ein wachsendes globales Publikum – alle sechzig Minuten, in mehreren Sprachen und Regionen.
+Für Marken, die für Integrität, Transparenz, Innovation und verantwortungsvolle künstliche Intelligenz stehen, bietet BalVoi:60 mehr als Werbung.
 Es bietet die Möglichkeit, gemeinsame Werte zu unterstützen.
 Erreichen Sie Menschen, die Fakten, fundierte Analysen und vertrauenswürdige Informationen schätzen.
 Erfahren Sie mehr über Sponsoring-Möglichkeiten auf BalVoi.com.
-BalVoi:30. Die ausgewogene Stimme der Nachrichten.</t>
+BalVoi:60. Die ausgewogene Stimme der Nachrichten.</t>
   </si>
   <si>
     <t>كل يوم، يتعرض ملايين الأشخاص لكمٍّ من المعلومات يفوق ما عرفه أي جيل سابق.
 لم تكن الثقة أكثر قيمة مما هي عليه اليوم.
-تقدم BalVoi:30 أخبارًا متوازنة وجديرة بالثقة لجمهور عالمي متنامٍ، مع تحديثات كل ثلاثين دقيقة عبر لغات ومناطق متعددة.
-بالنسبة للعلامات التجارية التي تؤمن بالنزاهة والشفافية والابتكار والذكاء الاصطناعي المسؤول، فإن BalVoi:30 تقدم أكثر من مجرد فرصة إعلانية.
+تقدم BalVoi:60 أخبارًا متوازنة وجديرة بالثقة لجمهور عالمي متنامٍ، مع تحديثات كل ستين دقيقة عبر لغات ومناطق متعددة.
+بالنسبة للعلامات التجارية التي تؤمن بالنزاهة والشفافية والابتكار والذكاء الاصطناعي المسؤول، فإن BalVoi:60 تقدم أكثر من مجرد فرصة إعلانية.
 إنها فرصة للارتباط بقيم مشتركة.
 تواصلوا مع جمهور يقدّر الحقائق والتحليل المدروس والمعلومات الموثوقة.
 للتعرف على فرص الرعاية، زوروا BalVoi.com.
-BalVoi:30. الصوت المتوازن في الأخبار.</t>
+BalVoi:60. الصوت المتوازن في الأخبار.</t>
+  </si>
+  <si>
+    <t>Her gün milyonlarca insan, tarihteki herhangi bir nesilden daha fazla bilgiye maruz kalıyor.
+Güven hiç bu kadar değerli olmamıştı.
+BalVoi:60, her altmış dakikada bir yayınlanan güncellemelerle, birden fazla dil ve bölgede büyüyen küresel bir kitleye dengeli ve güvenilir haberler sunmaktadır.
+Dürüstlük, şeffaflık, yenilikçilik ve sorumlu yapay zekâ değerlerine bağlı markalar için BalVoi:60 yalnızca bir reklam fırsatı değildir.
+Ortak değerlere dayalı bir iş birliği fırsatıdır.
+Gerçeklere, düşünceli analizlere ve güvenilir bilgiye değer veren kitlelerle buluşun.
+Sponsorluk fırsatları hakkında daha fazla bilgi için BalVoi.com'u ziyaret edin.
+BalVoi:60. Haberlerdeki dengeli ses.</t>
   </si>
   <si>
     <t>Каждый день миллионы людей сталкиваются с большим объёмом информации, чем когда-либо прежде.
 Доверие ещё никогда не было столь ценным.
-BalVoi:30 предоставляет сбалансированные и надёжные новости для растущей международной аудитории, предлагая обновления каждые тридцать минут на нескольких языках.
-Для брендов, которые ценят честность, прозрачность, инновации и ответственное использование искусственного интеллекта, BalVoi:30 — это больше, чем реклама.
+BalVoi:60 предоставляет сбалансированные и надёжные новости для растущей международной аудитории, предлагая обновления каждые шестьдесят минут на нескольких языках.
+Для брендов, которые ценят честность, прозрачность, инновации и ответственное использование искусственного интеллекта, BalVoi:60 — это больше, чем реклама.
 Это возможность поддержать общие ценности.
 Присоединяйтесь к аудитории, которая ценит факты, вдумчивый анализ и надёжную информацию.
 Узнайте больше о возможностях спонсорства на BalVoi.com.
-BalVoi:30. Сбалансированный голос новостей.</t>
-  </si>
-  <si>
-    <t>Her gün milyonlarca insan, tarihteki herhangi bir nesilden daha fazla bilgiye maruz kalıyor.
-Güven hiç bu kadar değerli olmamıştı.
-BalVoi:30, her otuz dakikada bir yayınlanan güncellemelerle, birden fazla dil ve bölgede büyüyen küresel bir kitleye dengeli ve güvenilir haberler sunmaktadır.
-Dürüstlük, şeffaflık, yenilikçilik ve sorumlu yapay zekâ değerlerine bağlı markalar için BalVoi:30 yalnızca bir reklam fırsatı değildir.
-Ortak değerlere dayalı bir iş birliği fırsatıdır.
-Gerçeklere, düşünceli analizlere ve güvenilir bilgiye değer veren kitlelerle buluşun.
-Sponsorluk fırsatları hakkında daha fazla bilgi için BalVoi.com'u ziyaret edin.
-BalVoi:30. Haberlerdeki dengeli ses.</t>
-  </si>
-  <si>
-    <t>What does your brand stand for?
-In a world of information overload, growing polarization, and declining trust, consumers increasingly support organizations that value transparency, trust, and accountability.
-BalVoi:30 is building a global network of multilingual news programming powered by NewsGenie technology and dedicated to trustworthy information and informed audiences.
-We invite mission-driven brands to join us.
-If your organization believes technology should strengthen understanding rather than division, and that trust is earned through action, we'd love to talk.
-Learn more about sponsorship opportunities at BalVoi.com.
-BalVoi:30. Trustworthy information for a connected world.</t>
-  </si>
-  <si>
-    <t>¿Qué representa su marca?
-En un mundo de sobrecarga informativa, creciente polarización y disminución de la confianza, los consumidores apoyan cada vez más a las organizaciones que valoran la transparencia, la confianza y la responsabilidad.
-BalVoi:30 está construyendo una red global de programación informativa multilingüe impulsada por la tecnología de NewsGenie y dedicada a la información confiable y a audiencias bien informadas.
-Invitamos a las marcas con propósito a unirse a nosotros.
-Si su organización cree que la tecnología debe fortalecer el entendimiento en lugar de la división, y que la confianza se gana con acciones, nos gustaría conversar.
-Obtenga más información sobre oportunidades de patrocinio en BalVoi.com.
-BalVoi:30. Información confiable para un mundo conectado.</t>
-  </si>
-  <si>
-    <t>O que a sua marca representa?
-Em um mundo de excesso de informação, crescente polarização e queda da confiança, os consumidores apoiam cada vez mais organizações que valorizam transparência, confiança e responsabilidade.
-A BalVoi:30 está construindo uma rede global de programação informativa multilíngue impulsionada pela tecnologia da NewsGenie e dedicada à informação confiável e a públicos bem informados.
-Convidamos marcas com propósito a se juntarem a nós.
-Se sua organização acredita que a tecnologia deve fortalecer a compreensão em vez da divisão, e que a confiança é conquistada por meio de ações, gostaríamos de conversar.
-Saiba mais sobre oportunidades de patrocínio em BalVoi.com.
-BalVoi:30. Informação confiável para um mundo conectado.</t>
-  </si>
-  <si>
-    <t>Que représente votre marque ?
-Dans un monde marqué par la surcharge d'information, une polarisation croissante et un recul de la confiance, les consommateurs soutiennent de plus en plus les organisations qui valorisent la transparence, la confiance et la responsabilité.
-BalVoi:30 construit un réseau mondial de programmes d'information multilingues alimenté par la technologie NewsGenie et dédié à une information fiable et à des audiences éclairées.
-Nous invitons les marques porteuses d'une mission à nous rejoindre.
-Si votre organisation croit que la technologie doit renforcer la compréhension plutôt que la division, et que la confiance se gagne par les actes, nous serions heureux d'échanger avec vous.
-Découvrez les opportunités de partenariat sur BalVoi.com.
-BalVoi:30. Une information fiable pour un monde connecté.</t>
-  </si>
-  <si>
-    <t>Wofür steht Ihre Marke?
-In einer Welt voller Informationsüberlastung, wachsender Polarisierung und schwindenden Vertrauens unterstützen Verbraucher zunehmend Organisationen, die Transparenz, Vertrauen und Verantwortung schätzen.
-BalVoi:30 baut ein globales Netzwerk mehrsprachiger Nachrichtenprogramme auf, das von der NewsGenie-Technologie unterstützt wird und sich vertrauenswürdigen Informationen sowie informierten Zielgruppen widmet.
-Wir laden werteorientierte Marken ein, Teil dieser Mission zu werden.
-Wenn Ihr Unternehmen daran glaubt, dass Technologie Verständnis fördern statt Spaltung vertiefen sollte und dass Vertrauen durch Taten verdient wird, würden wir uns gerne mit Ihnen austauschen.
-Erfahren Sie mehr über Sponsoring-Möglichkeiten auf BalVoi.com.
-BalVoi:30. Vertrauenswürdige Informationen für eine vernetzte Welt.</t>
-  </si>
-  <si>
-    <t>بماذا تُعرف علامتكم التجارية؟
-في عالم يشهد فيضًا من المعلومات وتزايدًا في الاستقطاب وتراجعًا في الثقة، يتجه المستهلكون بشكل متزايد نحو المؤسسات التي تؤمن بالشفافية والثقة والمساءلة.
-تبني BalVoi:30 شبكة عالمية من البرامج الإخبارية متعددة اللغات، مدعومة بتقنية NewsGenie ومكرسة لتقديم معلومات موثوقة لجمهور واعٍ ومطلع.
-ندعو العلامات التجارية ذات الرسالة الواضحة للانضمام إلينا.
-إذا كانت مؤسستكم تؤمن بأن التكنولوجيا يجب أن تعزز الفهم بدلاً من الانقسام، وأن الثقة تُكتسب من خلال الأفعال، فسيسعدنا التواصل معكم.
-تعرفوا على فرص الرعاية عبر BalVoi.com.
-BalVoi:30. معلومات موثوقة لعالم مترابط.</t>
-  </si>
-  <si>
-    <t>Что представляет собой ваш бренд?
-В мире информационной перегрузки, растущей поляризации и снижения уровня доверия люди всё чаще поддерживают организации, которые ценят прозрачность, доверие и ответственность.
-BalVoi:30 создаёт глобальную сеть многоязычных новостных программ на базе технологий NewsGenie, ориентированную на надёжную информацию и информированную аудиторию.
-Мы приглашаем бренды с миссией присоединиться к нам.
-Если ваша организация считает, что технологии должны укреплять взаимопонимание, а не усиливать разногласия, и что доверие заслуживается действиями, мы будем рады сотрудничеству.
-Узнайте больше о возможностях спонсорства на BalVoi.com.
-BalVoi:30. Надёжная информация для взаимосвязанного мира.</t>
-  </si>
-  <si>
-    <t>Markanız neyi temsil ediyor?
-Bilgi fazlalığının, artan kutuplaşmanın ve azalan güvenin yaşandığı bir dünyada, tüketiciler şeffaflık, güven ve hesap verebilirlik değerlerini benimseyen kuruluşları giderek daha fazla desteklemektedir.
-BalVoi:30, NewsGenie teknolojisiyle desteklenen ve güvenilir bilgi ile bilinçli kitlelere odaklanan çok dilli küresel bir haber ağı inşa etmektedir.
-Misyon sahibi markaları bize katılmaya davet ediyoruz.
-Kuruluşunuz teknolojinin ayrışmayı değil anlayışı güçlendirmesi gerektiğine ve güvenin eylemlerle kazanıldığına inanıyorsa, sizinle konuşmak isteriz.
-Sponsorluk fırsatları hakkında daha fazla bilgi için BalVoi.com'u ziyaret edin.
-BalVoi:30. Bağlantılı bir dünya için güvenilir bilgi.</t>
-  </si>
-  <si>
-    <t>Artificial intelligence is changing how the world creates, distributes, and consumes information.
-The question is not whether AI will shape the future.
-The question is how.
-BalVoi:30 partners with organizations that believe AI can be used responsibly to increase transparency, improve understanding, and strengthen public trust.
-Our multilingual information network reaches audiences across North America, Latin America, Europe, the Middle East, and Eurasia.
-If your brand believes in innovation with purpose, we invite you to join us.
-BalVoi:30.
-Global reach. Trustworthy information. Responsible AI.</t>
-  </si>
-  <si>
-    <t>La inteligencia artificial está transformando la forma en que el mundo crea, distribuye y consume información.
-La pregunta no es si la inteligencia artificial cambiará el futuro.
-La pregunta es cómo lo hará.
-BalVoi:30 colabora con organizaciones que creen que la inteligencia artificial puede utilizarse de manera responsable para aumentar la transparencia, mejorar el entendimiento y fortalecer la confianza pública.
-Nuestra red multilingüe de información conecta audiencias en América del Norte, América Latina, Europa, Oriente Medio y Eurasia.
-Si su organización cree en la innovación con propósito, queremos conocerla.
-BalVoi:30.
-Alcance global. Información confiable. Inteligencia artificial responsable.</t>
-  </si>
-  <si>
-    <t>A inteligência artificial está transformando a maneira como o mundo cria, distribui e consome informação.
-A questão não é se a inteligência artificial moldará o futuro.
-A questão é como.
-A BalVoi:30 trabalha com organizações que acreditam que a inteligência artificial pode ser usada de forma responsável para aumentar a transparência, melhorar a compreensão e fortalecer a confiança pública.
-Nossa rede multilíngue de informação conecta audiências na América do Norte, América Latina, Europa, Oriente Médio e Eurásia.
-Se sua organização acredita em inovação com propósito, queremos conversar.
-BalVoi:30.
-Alcance global. Informação confiável. Inteligência artificial responsável.</t>
-  </si>
-  <si>
-    <t>L'intelligence artificielle transforme la manière dont le monde crée, diffuse et consomme l'information.
-La question n'est pas de savoir si l'intelligence artificielle façonnera l'avenir.
-La question est de savoir comment.
-BalVoi:30 s'associe à des organisations qui croient que l'intelligence artificielle peut être utilisée de manière responsable pour renforcer la transparence, améliorer la compréhension et accroître la confiance du public.
-Notre réseau multilingue d'information rejoint des audiences en Amérique du Nord, en Amérique latine, en Europe, au Moyen-Orient et en Eurasie.
-Si votre organisation croit en une innovation porteuse de sens, nous aimerions échanger avec vous.
-BalVoi:30.
-Portée mondiale. Information digne de confiance. Intelligence artificielle responsable.</t>
-  </si>
-  <si>
-    <t>Künstliche Intelligenz verändert, wie die Welt Informationen erstellt, verbreitet und konsumiert.
-Die Frage ist nicht, ob künstliche Intelligenz die Zukunft prägen wird.
-Die Frage ist, wie.
-BalVoi:30 arbeitet mit Organisationen zusammen, die daran glauben, dass künstliche Intelligenz verantwortungsvoll eingesetzt werden kann, um Transparenz zu fördern, Verständnis zu verbessern und öffentliches Vertrauen zu stärken.
-Unser mehrsprachiges Informationsnetzwerk erreicht Zielgruppen in Nordamerika, Lateinamerika, Europa, dem Nahen Osten und Eurasien.
-Wenn Ihr Unternehmen an Innovation mit Verantwortung glaubt, würden wir gerne mit Ihnen sprechen.
-BalVoi:30.
-Globale Reichweite. Vertrauenswürdige Informationen. Verantwortungsvolle künstliche Intelligenz.</t>
-  </si>
-  <si>
-    <t>يُغيّر الذكاء الاصطناعي الطريقة التي يُنشئ بها العالم المعلومات ويوزعها ويستهلكها.
-السؤال ليس ما إذا كان الذكاء الاصطناعي سيشكل المستقبل.
-السؤال هو كيف.
-تتعاون BalVoi:30 مع المؤسسات التي تؤمن بأن الذكاء الاصطناعي يمكن استخدامه بمسؤولية لتعزيز الشفافية وتحسين الفهم وتقوية الثقة العامة.
-تصل شبكتنا متعددة اللغات للمعلومات إلى جماهير في أمريكا الشمالية وأمريكا اللاتينية وأوروبا والشرق الأوسط وأوراسيا.
-إذا كانت مؤسستكم تؤمن بالابتكار الهادف، فنحن ندعوكم للانضمام إلينا.
-BalVoi:30.
-انتشار عالمي. معلومات جديرة بالثقة. ذكاء اصطناعي مسؤول.</t>
-  </si>
-  <si>
-    <t>Искусственный интеллект меняет способы создания, распространения и потребления информации во всём мире.
-Вопрос не в том, повлияет ли искусственный интеллект на будущее.
-Вопрос в том, каким будет это влияние.
-BalVoi:30 сотрудничает с организациями, которые считают, что искусственный интеллект должен использоваться ответственно для повышения прозрачности, улучшения понимания происходящего и укрепления общественного доверия.
-Наша многоязычная информационная сеть объединяет аудитории в Северной Америке, Латинской Америке, Европе, на Ближнем Востоке и в Евразии.
-Если ваша организация верит в инновации со смыслом, мы будем рады сотрудничеству.
-BalVoi:30.
-Глобальный охват. Надёжная информация. Ответственный искусственный интеллект.</t>
-  </si>
-  <si>
-    <t>Yapay zekâ, dünyanın bilgiyi üretme, dağıtma ve tüketme biçimini değiştiriyor.
-Soru, yapay zekânın geleceği şekillendirip şekillendirmeyeceği değildir.
-Soru, bunu nasıl yapacağıdır.
-BalVoi:30; yapay zekânın şeffaflığı artırmak, anlayışı geliştirmek ve kamu güvenini güçlendirmek için sorumlu bir şekilde kullanılabileceğine inanan kuruluşlarla iş birliği yapmaktadır.
-Çok dilli bilgi ağımız Kuzey Amerika, Latin Amerika, Avrupa, Orta Doğu ve Avrasya'daki kitlelere ulaşmaktadır.
-Kuruluşunuz amaç odaklı inovasyona inanıyorsa, sizinle tanışmak isteriz.
-BalVoi:30.
-Küresel erişim. Güvenilir bilgi. Sorumlu yapay zekâ.</t>
-  </si>
-  <si>
-    <t>English Ad 2</t>
-  </si>
-  <si>
-    <t>Spanish Ad 2</t>
-  </si>
-  <si>
-    <t>Portuguese Ad 2</t>
-  </si>
-  <si>
-    <t>French Ad 2</t>
-  </si>
-  <si>
-    <t>German Ad 2</t>
-  </si>
-  <si>
-    <t>Arabic Ad 2</t>
-  </si>
-  <si>
-    <t>Russian Ad 2</t>
-  </si>
-  <si>
-    <t>Turkish Ad 2</t>
+BalVoi:60. Сбалансированный голос новостей.</t>
   </si>
 </sst>
 </file>
@@ -2408,7 +2408,7 @@
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="46.85546875" customWidth="1"/>
+    <col min="1" max="1" width="71.7109375" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="27.85546875" customWidth="1"/>
     <col min="4" max="4" width="30.5703125" customWidth="1"/>
@@ -2715,7 +2715,7 @@
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="47.7109375" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="27.85546875" customWidth="1"/>
     <col min="4" max="4" width="30.5703125" customWidth="1"/>
@@ -3160,54 +3160,54 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>422</v>
+        <v>398</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>423</v>
+        <v>399</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>424</v>
+        <v>400</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>425</v>
+        <v>401</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>426</v>
+        <v>402</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>427</v>
+        <v>403</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>428</v>
+        <v>404</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>429</v>
+        <v>405</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>398</v>
+        <v>422</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>399</v>
+        <v>423</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>400</v>
+        <v>424</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>401</v>
+        <v>425</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>402</v>
+        <v>426</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>403</v>
+        <v>427</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>404</v>
+        <v>429</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>405</v>
+        <v>428</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
@@ -3272,7 +3272,7 @@
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="42.85546875" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="27.85546875" customWidth="1"/>
     <col min="4" max="4" width="30.5703125" customWidth="1"/>

</xml_diff>

<commit_message>
BalVoi:60 — Megaphone publication path, settings validation, docs
</commit_message>
<xml_diff>
--- a/BalVoi_30 Content.xlsx
+++ b/BalVoi_30 Content.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{CAEBA2F1-DA58-4F11-BE30-1915A801D1A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FCC1C599-70E2-4D7E-8C9D-C286FBCB7CE0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="5" xr2:uid="{04BEA111-B2D1-43D4-8D75-B7B3005C7E34}"/>
+    <workbookView xWindow="9960" yWindow="1635" windowWidth="23580" windowHeight="9915" xr2:uid="{04BEA111-B2D1-43D4-8D75-B7B3005C7E34}"/>
   </bookViews>
   <sheets>
     <sheet name="Welcome" sheetId="7" r:id="rId1"/>
@@ -1706,6 +1706,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>